<commit_message>
Add AI service and documentation, update sample files
</commit_message>
<xml_diff>
--- a/sample_files/employee_data.xlsx
+++ b/sample_files/employee_data.xlsx
@@ -476,7 +476,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Robert Smith</t>
+          <t>Maria Davis</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,25 +486,25 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>829.889.5259</t>
+          <t>417.269.2075</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2024-10-06</t>
+          <t>02/02/2024</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>129536</v>
+        <v>146851</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Emma Smith</t>
+          <t>Michael Smith</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -524,7 +524,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>+1 (736)-231-9284</t>
+          <t>+1 (616)-909-4167</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -534,17 +534,17 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>07-Oct-2019</t>
+          <t>12/13/2017</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>$80,386</t>
+          <t>$92,173</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -554,7 +554,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Sarah Brown</t>
+          <t>Maria Smith</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -564,18 +564,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>+1 (518)-654-3012</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>+1 (594)-332-3714</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>06-Dec-2021</t>
+          <t>29-Jun-2017</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>$134,450</t>
+          <t>$102,329</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -600,27 +604,27 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>+1 (608)-816-2256</t>
+          <t>+1 (520)-578-8389</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2023-11-29</t>
+          <t>11-May-2024</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>$142,269</t>
+          <t>$133,936</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -630,7 +634,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sarah Johnson</t>
+          <t>Robert Brown</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -640,7 +644,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>+1 (973)-734-2096</t>
+          <t>+1 (396)-330-6489</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -650,17 +654,17 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>06/22/2019</t>
+          <t>12/21/2019</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>$77,401</t>
+          <t>$56,355</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -670,7 +674,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Robert Williams</t>
+          <t>Maria Jones</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -680,25 +684,25 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>+1 (539)-956-8289</t>
+          <t>+1 (635)-821-4999</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2025-04-01</t>
+          <t>25-Dec-2022</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>141970</v>
+        <v>66069</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -708,7 +712,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Michael Jones</t>
+          <t>Emma Williams</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -718,7 +722,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>503.613.9094</t>
+          <t>189.645.4805</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -728,12 +732,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2019-04-25</t>
+          <t>18-Sep-2017</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>$139,431</t>
+          <t>$34,107</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -748,7 +752,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Robert Smith</t>
+          <t>Emma Williams</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -758,22 +762,18 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>+1 (123)-889-6228</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Operations</t>
-        </is>
-      </c>
+          <t>+1 (222)-720-5822</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>07/30/2019</t>
+          <t>09/30/2019</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>$97,279</t>
+          <t>$46,793</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Robert Davis</t>
+          <t>Robert Smith</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -798,7 +798,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>+1 (625)-699-3724</t>
+          <t>+1 (952)-163-1548</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -808,17 +808,17 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>01/06/2020</t>
+          <t>20-Jan-2016</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>$75,443</t>
+          <t>$33,421</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -828,7 +828,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Maria Jones</t>
+          <t>John Johnson</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -838,27 +838,19 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>+1 (732)-942-7652</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
+          <t>+1 (683)-643-4509</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>06/02/2024</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>$62,506</t>
-        </is>
-      </c>
+          <t>2022-02-10</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -868,7 +860,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Sarah Jones</t>
+          <t>John Johnson</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -878,25 +870,21 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>+1 (498)-174-4779</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
+          <t>+1 (229)-614-4950</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>01/30/2020</t>
+          <t>2025-03-28</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>98331</v>
+        <v>92137</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -906,7 +894,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Michael Jones</t>
+          <t>Michael Johnson</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -916,23 +904,27 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>+1 (874)-688-5224</t>
+          <t>+1 (467)-659-7012</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>26-Mar-2018</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr"/>
+          <t>16-Apr-2023</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>$119,210</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -942,7 +934,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Maria Williams</t>
+          <t>Sarah Brown</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -952,27 +944,19 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>705.458.1564</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>04/28/2023</t>
-        </is>
-      </c>
+          <t>622.809.6637</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>$53,637</t>
+          <t>$121,677</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -982,37 +966,33 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Sarah Davis</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>employee_14@example.com</t>
-        </is>
-      </c>
+          <t>Michael Johnson</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>+1 (511)-552-8220</t>
+          <t>+1 (179)-820-2372</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>10-Dec-2023</t>
+          <t>10/27/2020</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>$91,731</t>
+          <t>$143,456</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1002,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Michael Brown</t>
+          <t>Emma Smith</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1032,27 +1012,27 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>+1 (427)-779-8474</t>
+          <t>+1 (636)-934-8942</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>08/14/2017</t>
+          <t>11/15/2016</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>$85,453</t>
+          <t>$105,655</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1042,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Maria Johnson</t>
+          <t>John Brown</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1072,25 +1052,25 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>+1 (689)-706-1640</t>
+          <t>+1 (296)-347-4508</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2024-03-03</t>
+          <t>24-Jun-2022</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>122067</v>
+        <v>69659</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1080,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Maria Jones</t>
+          <t>Emma Williams</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1110,22 +1090,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>+1 (569)-795-7395</t>
+          <t>+1 (827)-750-7408</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2023-03-07</t>
+          <t>02/18/2016</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>$140,982</t>
+          <t>$98,661</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1150,25 +1130,29 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>+1 (687)-259-1525</t>
+          <t>+1 (139)-945-6094</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>05-May-2015</t>
+          <t>2016-08-24</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>$98,859</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr"/>
+          <t>$40,867</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1176,7 +1160,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Emma Johnson</t>
+          <t>Michael Brown</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1186,27 +1170,27 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>381.225.7137</t>
+          <t>614.740.9425</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2024-08-29</t>
+          <t>2021-04-30</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>$43,828</t>
+          <t>$79,29</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1200,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Robert Williams</t>
+          <t>Emma Johnson</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1226,27 +1210,27 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>+1 (637)-801-9143</t>
+          <t>+1 (443)-926-5374</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>20-Dec-2021</t>
+          <t>2019-01-23</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>$122,723</t>
+          <t>$110,572</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1240,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>John Jones</t>
+          <t>Maria Johnson</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1266,23 +1250,27 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>+1 (375)-193-6367</t>
+          <t>+1 (386)-161-4892</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2025-02-07</t>
+          <t>15-Oct-2018</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>139562</v>
-      </c>
-      <c r="H22" t="inlineStr"/>
+        <v>111052</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1290,7 +1278,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Robert Brown</t>
+          <t>Michael Johnson</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1300,27 +1288,27 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>+1 (253)-620-1473</t>
+          <t>+1 (973)-113-8754</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2021-09-04</t>
+          <t>22-Feb-2023</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>$109,151</t>
+          <t>$98,615</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1328,11 +1316,7 @@
       <c r="A24" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Emma Smith</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>employee_23@example.com</t>
@@ -1340,7 +1324,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>+1 (933)-323-4504</t>
+          <t>+1 (409)-123-2928</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1350,17 +1334,17 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>12/25/2023</t>
+          <t>11/27/2018</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>$74,680</t>
+          <t>$78,193</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1354,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Robert Smith</t>
+          <t>Michael Williams</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1380,7 +1364,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>+1 (225)-212-2448</t>
+          <t>+1 (716)-267-9228</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1390,19 +1374,15 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>04/20/2019</t>
+          <t>21-Jul-2015</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>$117,502</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>$30,894</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1410,7 +1390,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Maria Jones</t>
+          <t>John Jones</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1418,25 +1398,29 @@
           <t>employee_25@example.com</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>343.616.2248</t>
+        </is>
+      </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2019-06-10</t>
+          <t>05/27/2021</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>$50,216</t>
+          <t>$125,834</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1446,7 +1430,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Michael Smith</t>
+          <t>Robert Davis</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1456,25 +1440,25 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>+1 (818)-682-1673</t>
+          <t>+1 (278)-297-1149</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>05/25/2017</t>
+          <t>2017-03-02</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>97035</v>
+        <v>95572</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1484,7 +1468,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Robert Williams</t>
+          <t>John Davis</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1494,25 +1478,25 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>+1 (392)-277-5054</t>
+          <t>+1 (942)-245-9495</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>02/18/2023</t>
-        </is>
-      </c>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>$32,189</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
+          <t>$66,238</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1520,7 +1504,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Sarah Johnson</t>
+          <t>Sarah Jones</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1530,23 +1514,27 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>+1 (785)-780-1519</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr"/>
+          <t>+1 (594)-473-1254</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>07/26/2024</t>
+          <t>03/04/2019</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>$98,956</t>
+          <t>$135,558</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -1556,13 +1544,13 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Sarah Johnson</t>
+          <t>John Brown</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>+1 (453)-962-8327</t>
+          <t>+1 (858)-224-6299</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1572,17 +1560,17 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>11/18/2021</t>
+          <t>14-Jul-2017</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>$79,0</t>
+          <t>$72,801</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1592,7 +1580,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Emma Brown</t>
+          <t>John Williams</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1602,27 +1590,27 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>+1 (955)-573-3543</t>
+          <t>+1 (880)-473-2712</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>09/16/2022</t>
+          <t>2018-09-02</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>$106,672</t>
+          <t>$88,777</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1632,7 +1620,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Robert Davis</t>
+          <t>Sarah Jones</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1642,25 +1630,25 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>432.371.2092</t>
+          <t>417.645.8470</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2018-04-14</t>
+          <t>2019-11-27</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>37273</v>
+        <v>131263</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1658,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Emma Williams</t>
+          <t>Michael Davis</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1680,27 +1668,27 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>+1 (244)-133-2308</t>
+          <t>+1 (842)-747-1285</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2018-10-31</t>
+          <t>13-Nov-2018</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>$130,844</t>
+          <t>$50,478</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1710,33 +1698,37 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Maria Johnson</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
+          <t>Emma Johnson</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>employee_33@example.com</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>+1 (659)-643-7363</t>
+          <t>+1 (740)-373-3392</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>10/02/2023</t>
+          <t>05/25/2018</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>$103,613</t>
+          <t>$104,798</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -1746,7 +1738,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Michael Johnson</t>
+          <t>Maria Brown</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1756,27 +1748,27 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>+1 (625)-463-9822</t>
+          <t>+1 (271)-507-4061</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2023-04-09</t>
+          <t>08/20/2024</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>$103,7</t>
+          <t>$147,499</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1786,7 +1778,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Maria Johnson</t>
+          <t>Maria Brown</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1794,25 +1786,29 @@
           <t>employee_35@example.com</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>+1 (690)-309-1856</t>
+        </is>
+      </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2021-07-22</t>
+          <t>2019-02-17</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>$34,158</t>
+          <t>$55,911</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1822,7 +1818,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>John Jones</t>
+          <t>John Davis</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1832,21 +1828,25 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>+1 (972)-768-4028</t>
+          <t>+1 (926)-680-2260</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr"/>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>06/03/2024</t>
+        </is>
+      </c>
       <c r="G37" t="n">
-        <v>71475</v>
+        <v>147382</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Robert Davis</t>
+          <t>Robert Smith</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1866,22 +1866,22 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>291.569.6690</t>
+          <t>145.607.7781</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>12-Nov-2021</t>
+          <t>07/29/2024</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>$58,837</t>
+          <t>$128,566</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -1896,7 +1896,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Emma Smith</t>
+          <t>Maria Davis</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1906,7 +1906,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>+1 (156)-962-4987</t>
+          <t>+1 (397)-638-7709</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1916,12 +1916,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2019-01-06</t>
+          <t>2022-12-02</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>$50,508</t>
+          <t>$63,669</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Sarah Williams</t>
+          <t>Emma Davis</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1946,27 +1946,27 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>+1 (195)-492-2555</t>
+          <t>+1 (925)-387-4287</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>06/13/2022</t>
+          <t>15-Dec-2021</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>$123,717</t>
+          <t>$140,85</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1976,7 +1976,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>John Brown</t>
+          <t>Emma Jones</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1986,27 +1986,27 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>+1 (695)-748-6912</t>
+          <t>+1 (751)-235-8957</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>06-Sep-2019</t>
+          <t>2016-12-20</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>$115,996</t>
+          <t>$104,658</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Michael Johnson</t>
+          <t>Emma Johnson</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2026,25 +2026,25 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>+1 (652)-908-9043</t>
+          <t>+1 (839)-487-7575</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2019-12-04</t>
+          <t>11-Feb-2021</t>
         </is>
       </c>
       <c r="G42" t="n">
-        <v>87929</v>
+        <v>90636</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2054,7 +2054,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Sarah Williams</t>
+          <t>Robert Davis</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2064,23 +2064,27 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>+1 (964)-652-5097</t>
+          <t>+1 (718)-136-7048</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2017-07-24</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr"/>
+          <t>04/05/2017</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>$104,199</t>
+        </is>
+      </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2090,7 +2094,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Maria Brown</t>
+          <t>John Brown</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2100,27 +2104,27 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>655.606.9390</t>
+          <t>519.383.1371</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2020-05-05</t>
+          <t>12/13/2023</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>$148,740</t>
+          <t>$40,795</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2130,7 +2134,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Emma Jones</t>
+          <t>Emma Williams</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2140,27 +2144,27 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>+1 (366)-516-1907</t>
+          <t>+1 (778)-811-7637</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>03-Mar-2023</t>
+          <t>2022-12-25</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>$89,977</t>
+          <t>$71,402</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2170,7 +2174,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Emma Johnson</t>
+          <t>Sarah Davis</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2180,27 +2184,27 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>+1 (907)-982-7699</t>
+          <t>+1 (108)-550-1017</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2021-08-12</t>
+          <t>02/18/2019</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>$49,169</t>
+          <t>$51,970</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -2210,7 +2214,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Sarah Johnson</t>
+          <t>Michael Jones</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2218,11 +2222,7 @@
           <t>employee_46@example.com</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>+1 (910)-413-3138</t>
-        </is>
-      </c>
+      <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
           <t>IT</t>
@@ -2230,15 +2230,15 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>15-Jun-2018</t>
+          <t>24-Sep-2024</t>
         </is>
       </c>
       <c r="G47" t="n">
-        <v>110716</v>
+        <v>84414</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2248,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Robert Williams</t>
+          <t>Sarah Johnson</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2258,29 +2258,25 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>+1 (807)-713-5776</t>
+          <t>+1 (299)-813-7324</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2019-12-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>$124,250</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>$97,303</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2288,7 +2284,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Sarah Williams</t>
+          <t>Maria Davis</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2298,27 +2294,23 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>+1 (121)-178-2632</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
+          <t>+1 (862)-593-6614</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
-          <t>03/20/2023</t>
+          <t>22-Sep-2024</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>$106,98</t>
+          <t>$78,762</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2320,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Robert Williams</t>
+          <t>Maria Jones</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2338,23 +2330,27 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>826.582.1846</t>
+          <t>190.450.5635</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr"/>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>13-Oct-2018</t>
+        </is>
+      </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>$142,762</t>
+          <t>$54,659</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2364,7 +2360,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>John Brown</t>
+          <t>John Jones</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2374,27 +2370,27 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>+1 (492)-365-6826</t>
+          <t>+1 (796)-536-3346</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2024-07-15</t>
+          <t>2021-11-22</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>$38,581</t>
+          <t>$92,121</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2400,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Sarah Johnson</t>
+          <t>Sarah Smith</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2414,25 +2410,25 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>+1 (419)-961-2162</t>
+          <t>+1 (905)-395-6116</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>11/19/2020</t>
+          <t>08/16/2017</t>
         </is>
       </c>
       <c r="G52" t="n">
-        <v>97647</v>
+        <v>80676</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -2442,7 +2438,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Michael Jones</t>
+          <t>Michael Brown</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2452,27 +2448,27 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>+1 (300)-238-2690</t>
+          <t>+1 (763)-254-7374</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>11-Nov-2020</t>
+          <t>11/06/2015</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>$82,215</t>
+          <t>$39,672</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2482,7 +2478,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Maria Johnson</t>
+          <t>Robert Davis</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2492,27 +2488,27 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>+1 (147)-282-7659</t>
+          <t>+1 (248)-184-8491</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>21-Jun-2022</t>
+          <t>07/25/2015</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>$101,534</t>
+          <t>$48,554</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2518,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>John Williams</t>
+          <t>Emma Johnson</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2532,29 +2528,25 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>+1 (213)-236-7925</t>
+          <t>+1 (445)-345-7046</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>02-Nov-2022</t>
+          <t>2023-01-06</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>$74,402</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+          <t>$95,266</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2562,7 +2554,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Sarah Smith</t>
+          <t>John Johnson</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2572,27 +2564,27 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>850.944.5289</t>
+          <t>931.111.3306</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2019-08-31</t>
+          <t>2022-03-09</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>$142,216</t>
+          <t>$49,794</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2602,7 +2594,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Michael Brown</t>
+          <t>Maria Smith</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2610,7 +2602,11 @@
           <t>employee_56@example.com</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>+1 (256)-897-5430</t>
+        </is>
+      </c>
       <c r="E57" t="inlineStr">
         <is>
           <t>IT</t>
@@ -2618,13 +2614,17 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>12/14/2023</t>
+          <t>20-Jul-2019</t>
         </is>
       </c>
       <c r="G57" t="n">
-        <v>148619</v>
-      </c>
-      <c r="H57" t="inlineStr"/>
+        <v>136073</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2632,7 +2632,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>John Davis</t>
+          <t>Maria Johnson</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2642,27 +2642,27 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>+1 (230)-716-1113</t>
+          <t>+1 (315)-790-9532</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>12/03/2018</t>
+          <t>21-Apr-2025</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>$78,331</t>
+          <t>$78,673</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -2682,23 +2682,27 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>+1 (807)-877-5575</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr"/>
+          <t>+1 (772)-434-2359</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>24-May-2023</t>
+          <t>09/10/2015</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>$149,49</t>
+          <t>$91,960</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2708,7 +2712,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Maria Williams</t>
+          <t>Robert Jones</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2718,24 +2722,20 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>+1 (726)-186-2781</t>
+          <t>+1 (444)-257-3287</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>2016-04-15</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>$108,108</t>
-        </is>
-      </c>
+          <t>11/24/2019</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2748,7 +2748,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Maria Williams</t>
+          <t>Maria Brown</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2758,22 +2758,22 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>+1 (356)-422-2119</t>
+          <t>+1 (161)-226-7200</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>03-Oct-2020</t>
+          <t>01/08/2016</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>$31,543</t>
+          <t>$126,364</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Emma Smith</t>
+          <t>Emma Williams</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2798,25 +2798,25 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>428.534.1034</t>
+          <t>848.751.8331</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>04-Dec-2022</t>
+          <t>2019-10-01</t>
         </is>
       </c>
       <c r="G62" t="n">
-        <v>60896</v>
+        <v>43071</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Michael Smith</t>
+          <t>Michael Davis</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2834,25 +2834,25 @@
           <t>employee_62@example.com</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr"/>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>+1 (121)-248-5463</t>
+        </is>
+      </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Operations</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>2019-05-24</t>
-        </is>
-      </c>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>$55,944</t>
+          <t>$50,490</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -2862,7 +2862,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>John Davis</t>
+          <t>Maria Williams</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2872,27 +2872,27 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>+1 (878)-947-7149</t>
+          <t>+1 (739)-752-3037</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>09/26/2021</t>
+          <t>2025-01-12</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>$124,549</t>
+          <t>$91,321</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2902,7 +2902,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Maria Smith</t>
+          <t>Robert Brown</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>+1 (306)-692-9731</t>
+          <t>+1 (176)-430-6505</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2920,15 +2920,19 @@
           <t>Sales</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>03/25/2023</t>
+        </is>
+      </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>$115,537</t>
+          <t>$39,208</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -2938,7 +2942,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Michael Williams</t>
+          <t>Maria Johnson</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2948,27 +2952,27 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>+1 (255)-736-7472</t>
+          <t>+1 (920)-570-5219</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>2019-06-27</t>
+          <t>2021-08-18</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>$108,717</t>
+          <t>$125,375</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -2978,7 +2982,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>John Brown</t>
+          <t>Sarah Johnson</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2988,21 +2992,17 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>+1 (627)-237-4550</t>
+          <t>+1 (473)-850-6422</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>24-Oct-2017</t>
-        </is>
-      </c>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
       <c r="G67" t="n">
-        <v>83791</v>
+        <v>54117</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Robert Brown</t>
+          <t>Michael Brown</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3026,27 +3026,23 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>123.498.9322</t>
+          <t>721.945.2012</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>2021-06-14</t>
-        </is>
-      </c>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>$118,290</t>
+          <t>$114,403</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -3056,7 +3052,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Sarah Brown</t>
+          <t>Emma Jones</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3066,23 +3062,27 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>+1 (491)-215-3044</t>
+          <t>+1 (395)-825-9280</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>04/11/2019</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr"/>
+          <t>02/01/2019</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>$125,934</t>
+        </is>
+      </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -3092,7 +3092,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Maria Jones</t>
+          <t>Robert Davis</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3102,27 +3102,27 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>+1 (555)-216-1137</t>
+          <t>+1 (513)-285-2031</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>2024-09-16</t>
+          <t>2020-05-30</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>$46,673</t>
+          <t>$121,926</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Emma Smith</t>
+          <t>John Johnson</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3142,27 +3142,27 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>+1 (823)-112-2211</t>
+          <t>+1 (776)-346-4625</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>29-Jun-2015</t>
+          <t>11/19/2023</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>$120,861</t>
+          <t>$130,184</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -3172,7 +3172,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Michael Brown</t>
+          <t>John Williams</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3182,7 +3182,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>+1 (269)-985-1996</t>
+          <t>+1 (398)-291-6287</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3192,15 +3192,15 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>31-May-2020</t>
+          <t>2023-01-06</t>
         </is>
       </c>
       <c r="G72" t="n">
-        <v>133495</v>
+        <v>61479</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Emma Johnson</t>
+          <t>John Jones</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3220,27 +3220,27 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>+1 (655)-758-2781</t>
+          <t>+1 (937)-313-8038</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>2021-06-21</t>
+          <t>17-Feb-2016</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>$131,661</t>
+          <t>$132,84</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -3250,17 +3250,13 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Michael Johnson</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>employee_73@example.com</t>
-        </is>
-      </c>
+          <t>John Brown</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr"/>
       <c r="D74" t="inlineStr">
         <is>
-          <t>329.487.7144</t>
+          <t>788.514.9838</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3270,17 +3266,17 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>2020-04-07</t>
+          <t>2018-12-01</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>$80,950</t>
+          <t>$34,71</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -3290,7 +3286,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>John Smith</t>
+          <t>Sarah Davis</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3300,27 +3296,27 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>+1 (307)-500-4559</t>
+          <t>+1 (291)-190-1270</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>16-Apr-2024</t>
+          <t>2016-06-10</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>$44,571</t>
+          <t>$110,390</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -3330,37 +3326,29 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>John Williams</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>employee_75@example.com</t>
-        </is>
-      </c>
+          <t>Michael Williams</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr"/>
       <c r="D76" t="inlineStr">
         <is>
-          <t>+1 (778)-227-7970</t>
+          <t>+1 (217)-721-8602</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>2017-10-13</t>
-        </is>
-      </c>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>$107,916</t>
+          <t>$147,406</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -3370,7 +3358,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Maria Williams</t>
+          <t>Sarah Jones</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3380,25 +3368,25 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>+1 (714)-395-9635</t>
+          <t>+1 (677)-516-2886</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>2016-07-01</t>
+          <t>11/08/2022</t>
         </is>
       </c>
       <c r="G77" t="n">
-        <v>133553</v>
+        <v>129062</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3408,7 +3396,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Robert Brown</t>
+          <t>Emma Davis</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3418,27 +3406,27 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>+1 (130)-941-5980</t>
+          <t>+1 (358)-691-2076</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>2021-08-13</t>
+          <t>2019-10-24</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>$106,85</t>
+          <t>$78,729</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -3448,7 +3436,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Sarah Jones</t>
+          <t>Maria Smith</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3458,27 +3446,27 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>+1 (919)-646-2278</t>
+          <t>+1 (875)-508-2373</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>11-Mar-2025</t>
+          <t>05/11/2025</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>$130,129</t>
+          <t>$55,602</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -3488,7 +3476,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Maria Williams</t>
+          <t>Emma Davis</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3498,27 +3486,27 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>505.150.7981</t>
+          <t>626.822.6290</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>09/06/2022</t>
+          <t>2024-01-31</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>$111,883</t>
+          <t>$55,316</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -3528,33 +3516,37 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Emma Davis</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr"/>
+          <t>Maria Williams</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>EMPLOYEE_80@EXAMPLE.COM</t>
+        </is>
+      </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>+1 (270)-455-4147</t>
+          <t>+1 (337)-185-7545</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>2022-07-29</t>
+          <t>02/25/2018</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>$36,732</t>
+          <t>$99,485</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -3564,7 +3556,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>John Jones</t>
+          <t>Sarah Williams</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3574,25 +3566,25 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>+1 (918)-233-7642</t>
+          <t>+1 (767)-932-4559</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>08/20/2018</t>
+          <t>2019-09-13</t>
         </is>
       </c>
       <c r="G82" t="n">
-        <v>81682</v>
+        <v>133727</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -3602,7 +3594,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Maria Jones</t>
+          <t>Sarah Smith</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3612,29 +3604,25 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>+1 (178)-773-9668</t>
+          <t>+1 (554)-136-1496</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>02-Jun-2022</t>
+          <t>2015-07-04</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>$32,194</t>
-        </is>
-      </c>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>$114,365</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -3642,7 +3630,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Robert Smith</t>
+          <t>Michael Davis</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -3652,27 +3640,27 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>+1 (947)-568-2970</t>
+          <t>+1 (402)-506-6194</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>04/27/2024</t>
+          <t>02/28/2021</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>$59,651</t>
+          <t>$141,380</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3682,7 +3670,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Sarah Brown</t>
+          <t>Robert Williams</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -3692,27 +3680,27 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>+1 (432)-319-4623</t>
+          <t>+1 (931)-349-6832</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>12/28/2024</t>
+          <t>2020-01-31</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>$63,494</t>
+          <t>$110,750</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -3722,7 +3710,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Robert Jones</t>
+          <t>Michael Davis</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -3732,27 +3720,27 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>856.960.4928</t>
+          <t>649.392.1856</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>12-Oct-2018</t>
+          <t>2023-03-01</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>$133,115</t>
+          <t>$113,123</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -3762,7 +3750,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Robert Johnson</t>
+          <t>John Brown</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -3772,25 +3760,25 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>+1 (167)-185-1910</t>
+          <t>+1 (273)-570-7403</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>2024-05-10</t>
+          <t>2022-06-07</t>
         </is>
       </c>
       <c r="G87" t="n">
-        <v>76666</v>
+        <v>50625</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -3798,7 +3786,11 @@
       <c r="A88" t="n">
         <v>87</v>
       </c>
-      <c r="B88" t="inlineStr"/>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Robert Williams</t>
+        </is>
+      </c>
       <c r="C88" t="inlineStr">
         <is>
           <t>employee_87@example.com</t>
@@ -3806,27 +3798,27 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>+1 (830)-941-1733</t>
+          <t>+1 (591)-829-5480</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>01/20/2018</t>
+          <t>2020-05-13</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>$108,714</t>
+          <t>$132,741</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -3836,7 +3828,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Maria Brown</t>
+          <t>Emma Jones</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -3846,23 +3838,27 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>+1 (894)-753-1311</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr"/>
+          <t>+1 (833)-121-8838</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>03/01/2019</t>
+          <t>10/10/2024</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>$109,923</t>
+          <t>$144,410</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3872,7 +3868,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Sarah Davis</t>
+          <t>Maria Davis</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -3882,27 +3878,23 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>+1 (407)-963-3205</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>Operations</t>
-        </is>
-      </c>
+          <t>+1 (935)-792-4574</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
-          <t>18-Feb-2017</t>
+          <t>24-Aug-2017</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>$100,310</t>
+          <t>$90,574</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -3912,7 +3904,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Michael Johnson</t>
+          <t>Sarah Jones</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -3922,27 +3914,23 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>+1 (571)-845-3712</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
+          <t>+1 (483)-741-4523</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
-          <t>2021-04-18</t>
+          <t>2023-11-06</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>$65,624</t>
+          <t>$62,239</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -3952,7 +3940,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Michael Brown</t>
+          <t>Sarah Williams</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -3962,25 +3950,25 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>732.982.2663</t>
+          <t>226.856.8390</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>24-Jan-2021</t>
+          <t>04/08/2023</t>
         </is>
       </c>
       <c r="G92" t="n">
-        <v>90654</v>
+        <v>88849</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -3990,7 +3978,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Maria Johnson</t>
+          <t>Emma Williams</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -4000,7 +3988,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>+1 (471)-991-4487</t>
+          <t>+1 (706)-281-6876</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4010,17 +3998,17 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>01/06/2020</t>
+          <t>2017-10-31</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>$117,885</t>
+          <t>$61,243</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -4030,7 +4018,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Robert Williams</t>
+          <t>Michael Jones</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -4040,7 +4028,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>+1 (723)-393-8570</t>
+          <t>+1 (668)-477-3138</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4050,17 +4038,17 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>08/28/2024</t>
+          <t>2022-01-15</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>$113,213</t>
+          <t>$33,48</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -4070,7 +4058,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Robert Jones</t>
+          <t>Emma Johnson</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -4080,7 +4068,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>+1 (572)-954-8986</t>
+          <t>+1 (732)-153-8266</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4090,17 +4078,17 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>13-Aug-2022</t>
+          <t>03/25/2018</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>$79,543</t>
+          <t>$66,820</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -4110,7 +4098,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Emma Williams</t>
+          <t>Michael Jones</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -4120,27 +4108,27 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>+1 (479)-299-1865</t>
+          <t>+1 (352)-611-9645</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>08/02/2023</t>
+          <t>20-Apr-2022</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>$58,495</t>
+          <t>$34,675</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4138,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Robert Johnson</t>
+          <t>Robert Davis</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -4160,25 +4148,25 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>+1 (705)-931-6323</t>
+          <t>+1 (936)-218-8977</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>2021-08-10</t>
+          <t>04/21/2023</t>
         </is>
       </c>
       <c r="G97" t="n">
-        <v>110140</v>
+        <v>38286</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4176,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Michael Williams</t>
+          <t>Robert Williams</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -4198,7 +4186,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>892.814.3647</t>
+          <t>206.796.6019</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -4208,17 +4196,17 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>19-May-2015</t>
+          <t>2018-10-03</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>$33,28</t>
+          <t>$78,54</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -4228,7 +4216,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>John Davis</t>
+          <t>Michael Brown</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -4238,27 +4226,27 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>+1 (116)-815-1028</t>
+          <t>+1 (267)-236-1018</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>05-Sep-2021</t>
+          <t>13-Feb-2018</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>$84,942</t>
+          <t>$76,177</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -4268,7 +4256,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Sarah Brown</t>
+          <t>Maria Brown</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -4278,27 +4266,27 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>+1 (913)-715-1084</t>
+          <t>+1 (184)-805-4087</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2020-11-28</t>
+          <t>25-May-2023</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>$90,531</t>
+          <t>$119,637</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -4308,7 +4296,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Emma Johnson</t>
+          <t>Robert Brown</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -4318,22 +4306,22 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>+1 (457)-122-6269</t>
+          <t>+1 (259)-786-4563</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>23-Sep-2023</t>
+          <t>04/03/2025</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>$44,866</t>
+          <t>$55,996</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">

</xml_diff>